<commit_message>
Mise à jour v24
</commit_message>
<xml_diff>
--- a/config/configuration-resultat.xlsx
+++ b/config/configuration-resultat.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tuto" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sport" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Équipes favorites" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Actus" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Actus International" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Marchés" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Vidéos" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="YouTube" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Programme TV" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Cotes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Accueil" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Apparence" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuto" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sport" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Équipes favorites" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actus" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actus International" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marchés" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidéos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programme TV" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accueil" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applis" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apparence" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sport'!$B$5:$K$157</definedName>
@@ -30,9 +31,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Vidéos'!$B$5:$J$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'YouTube'!$B$5:$G$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Programme TV'!$B$5:$G$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Cotes'!$B$5:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Cotes'!$B$5:$H$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Accueil'!$B$5:$G$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Apparence'!$B$5:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Applis'!$B$5:$I$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Apparence'!$B$5:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -884,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="39" min="1" max="1"/>
@@ -896,7 +898,7 @@
     <row r="1" ht="36" customHeight="1" s="40">
       <c r="B1" s="41" t="inlineStr">
         <is>
-          <t>Mon Écran · classeur de configuration (version 1)</t>
+          <t>Mon Écran · classeur de configuration (version 2)</t>
         </is>
       </c>
     </row>
@@ -1254,11 +1256,11 @@
         </is>
       </c>
       <c r="C37" s="50">
-        <f>COUNTIFS(Cotes!$F$6:$F$40,"Oui",Cotes!$A$6:$A$40,"&lt;&gt;sec:*")</f>
+        <f>COUNTIFS(Cotes!$F$6:$F$48,"Oui",Cotes!$A$6:$A$48,"&lt;&gt;sec:*")</f>
         <v/>
       </c>
       <c r="D37" s="50">
-        <f>COUNTIFS(Cotes!$A$6:$A$40,"&lt;&gt;sec:*",Cotes!$A$6:$A$40,"&lt;&gt;")</f>
+        <f>COUNTIFS(Cotes!$A$6:$A$48,"&lt;&gt;sec:*",Cotes!$A$6:$A$48,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="E37" s="51" t="inlineStr">
@@ -1290,69 +1292,107 @@
     <row r="39" ht="15" customHeight="1" s="40">
       <c r="B39" s="49" t="inlineStr">
         <is>
+          <t>Applis</t>
+        </is>
+      </c>
+      <c r="C39" s="50">
+        <f>COUNTIFS(Applis!$G$6:$G$54,"Oui",Applis!$A$6:$A$54,"&lt;&gt;sec:*")</f>
+        <v/>
+      </c>
+      <c r="D39" s="50">
+        <f>COUNTIFS(Applis!$A$6:$A$54,"&lt;&gt;sec:*",Applis!$A$6:$A$54,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="E39" s="51" t="inlineStr">
+        <is>
+          <t>Accueil · applis, dossiers et liens</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="40">
+      <c r="B40" s="49" t="inlineStr">
+        <is>
           <t>Apparence</t>
         </is>
       </c>
-      <c r="C39" s="50">
+      <c r="C40" s="50">
         <f>COUNTIFS(Apparence!$E$6:$E$17,"Oui",Apparence!$A$6:$A$17,"&lt;&gt;sec:*")</f>
         <v/>
       </c>
-      <c r="D39" s="50">
+      <c r="D40" s="50">
         <f>COUNTIFS(Apparence!$A$6:$A$17,"&lt;&gt;sec:*",Apparence!$A$6:$A$17,"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="E39" s="51" t="inlineStr">
+      <c r="E40" s="51" t="inlineStr">
         <is>
           <t>Apparence · thèmes et mode</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1" s="40">
-      <c r="B40" s="52" t="inlineStr">
+    <row r="41" ht="15" customHeight="1" s="40">
+      <c r="B41" s="52" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C40" s="52">
-        <f>SUM(C29:C39)</f>
+      <c r="C41" s="52">
+        <f>SUM(C29:C40)</f>
         <v/>
       </c>
-      <c r="D40" s="52">
-        <f>SUM(D29:D39)</f>
+      <c r="D41" s="52">
+        <f>SUM(D29:D40)</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1" s="40">
-      <c r="B42" s="42" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="40">
+      <c r="B43" s="42" t="inlineStr">
         <is>
           <t>Journal des versions du classeur</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="30" customHeight="1" s="40">
-      <c r="B43" s="52" t="inlineStr">
+    <row r="44" ht="30" customHeight="1" s="40">
+      <c r="B44" s="52" t="inlineStr">
         <is>
           <t>Version 1</t>
         </is>
       </c>
-      <c r="C43" s="53" t="inlineStr">
+      <c r="C44" s="53" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="D43" s="43" t="inlineStr">
+      <c r="D44" s="43" t="inlineStr">
         <is>
           <t>Première version : 11 onglets (Sport, Équipes favorites, Actus, Actus International, Marchés, Vidéos, YouTube, Programme TV, Cotes, Accueil, Apparence), pré-cochés à l'identique du dock actuel, catalogue de plus de 500 éléments à essayer, blocs « Mes ajouts », Tuto.</t>
         </is>
       </c>
     </row>
+    <row r="45" ht="30" customHeight="1" s="40">
+      <c r="B45" s="52" t="inlineStr">
+        <is>
+          <t>Version 2</t>
+        </is>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="D45" s="43" t="inlineStr">
+        <is>
+          <t>Onglet Applis : dossiers, bandeau du bas et navigation, avec 3 liens par appli (iPhone, Android, web) modifiables. Onglet Cotes : réglages du rapport des écarts. Les pages lisent désormais ces réglages (config/config.js).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B5:E5"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="B16:E16"/>
@@ -1360,11 +1400,10 @@
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B43:E43"/>
     <mergeCell ref="B12:E12"/>
-    <mergeCell ref="D43:E43"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B42:E42"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="B17:E17"/>
@@ -1373,6 +1412,7 @@
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B10:E10"/>
+    <mergeCell ref="D44:E44"/>
     <mergeCell ref="C25:E25"/>
   </mergeCells>
   <hyperlinks>
@@ -1386,7 +1426,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" location="'Programme%20TV'!B1" display="Programme TV" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" location="'Cotes'!B1" display="Cotes" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" location="'Accueil'!B1" display="Accueil" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" location="'Apparence'!B1" display="Apparence" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" location="'Applis'!B1" display="Applis" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" location="'Apparence'!B1" display="Apparence" r:id="rId12"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1417,7 +1458,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=tv;version=1</t>
+          <t>module=tv;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -4466,7 +4507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="1"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" style="39" min="1" max="1"/>
@@ -4483,7 +4524,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=cotes;version=1</t>
+          <t>module=cotes;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -4856,7 +4897,7 @@
       <c r="H14" s="72" t="n"/>
       <c r="I14" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "fra.1", "cle": "soccer_france_ligue_one", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "fra.1", "cle": "soccer_france_ligue_one", "re": {"re": "ligue 1", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4936,7 @@
       <c r="H15" s="72" t="n"/>
       <c r="I15" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "eng.1", "cle": "soccer_epl", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "eng.1", "cle": "soccer_epl", "re": {"re": "^epl$|premier league", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4975,7 @@
       <c r="H16" s="72" t="n"/>
       <c r="I16" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "esp.1", "cle": "soccer_spain_la_liga", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "esp.1", "cle": "soccer_spain_la_liga", "re": {"re": "la ?liga", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -4973,7 +5014,7 @@
       <c r="H17" s="72" t="n"/>
       <c r="I17" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "ita.1", "cle": "soccer_italy_serie_a", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "ita.1", "cle": "soccer_italy_serie_a", "re": {"re": "serie a", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5053,7 @@
       <c r="H18" s="72" t="n"/>
       <c r="I18" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "ger.1", "cle": "soccer_germany_bundesliga", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "ger.1", "cle": "soccer_germany_bundesliga", "re": {"re": "^bundesliga(?! 2)", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5092,7 @@
       <c r="H19" s="72" t="n"/>
       <c r="I19" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "uefa.champions", "cle": "soccer_uefa_champs_league", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "uefa.champions", "cle": "soccer_uefa_champs_league", "re": {"re": "champions league(?!.*qualif)", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5131,7 @@
       <c r="H20" s="72" t="n"/>
       <c r="I20" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "uefa.europa", "cle": "soccer_uefa_europa_league", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "uefa.europa", "cle": "soccer_uefa_europa_league", "re": {"re": "europa league", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5170,7 @@
       <c r="H21" s="72" t="n"/>
       <c r="I21" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "uefa.europa.conf", "cle": "soccer_uefa_europa_conference_league", "re": {}}}</t>
+          <t>{"support": "ok", "def": {"id": "uefa.europa.conf", "cle": "soccer_uefa_europa_conference_league", "re": {"re": "conference league", "flags": "i"}}}</t>
         </is>
       </c>
     </row>
@@ -5874,171 +5915,315 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43" ht="15" customHeight="1" s="40">
-      <c r="B43" s="73" t="inlineStr">
-        <is>
-          <t>MES AJOUTS — tape ce que tu veux ajouter : la tâche essaie de le récupérer et écrit le résultat (✅ / ⚠️ / ❌) dans la colonne « Résultat »</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1" s="40">
-      <c r="B44" s="74" t="inlineStr">
-        <is>
-          <t>Section (Sites de paris ou Compétitions relevées)</t>
-        </is>
-      </c>
-      <c r="C44" s="74" t="inlineStr">
-        <is>
-          <t>Nom</t>
-        </is>
-      </c>
-      <c r="D44" s="74" t="inlineStr">
-        <is>
-          <t>Clé The Odds API ou id de compétition du dock</t>
-        </is>
-      </c>
-      <c r="F44" s="74" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="G44" s="74" t="inlineStr">
-        <is>
-          <t>Résultat</t>
-        </is>
-      </c>
-      <c r="H44" s="74" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="40">
+    <row r="41" ht="15" customHeight="1" s="40">
+      <c r="A41" s="39" t="inlineStr">
+        <is>
+          <t>sec:cotes:rapport_seuil</t>
+        </is>
+      </c>
+      <c r="B41" s="66" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · seuil d'affichage (un seul)</t>
+        </is>
+      </c>
+      <c r="C41" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D41" s="68" t="n"/>
+      <c r="E41" s="68" t="n"/>
+      <c r="F41" s="69" t="n"/>
+      <c r="G41" s="68" t="n"/>
+      <c r="H41" s="68" t="n"/>
+      <c r="I41" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "rapport_seuil", "label": "Rapport des écarts · seuil d'affichage (un seul)"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A42" s="39" t="inlineStr">
+        <is>
+          <t>cr:seuil:3</t>
+        </is>
+      </c>
+      <c r="B42" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · seuil d'affichage (un seul)</t>
+        </is>
+      </c>
+      <c r="C42" s="71" t="inlineStr">
+        <is>
+          <t>Écart d'au moins 3 %</t>
+        </is>
+      </c>
+      <c r="D42" s="71" t="n"/>
+      <c r="E42" s="71" t="n"/>
+      <c r="F42" s="69" t="n"/>
+      <c r="G42" s="72" t="n"/>
+      <c r="H42" s="72" t="n"/>
+      <c r="I42" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": 0.03}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A43" s="39" t="inlineStr">
+        <is>
+          <t>cr:seuil:5</t>
+        </is>
+      </c>
+      <c r="B43" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · seuil d'affichage (un seul)</t>
+        </is>
+      </c>
+      <c r="C43" s="71" t="inlineStr">
+        <is>
+          <t>Écart d'au moins 5 %</t>
+        </is>
+      </c>
+      <c r="D43" s="71" t="n"/>
+      <c r="E43" s="71" t="n"/>
+      <c r="F43" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G43" s="72" t="n"/>
+      <c r="H43" s="72" t="n"/>
+      <c r="I43" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": 0.05}</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>cr:seuil:8</t>
+        </is>
+      </c>
+      <c r="B44" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · seuil d'affichage (un seul)</t>
+        </is>
+      </c>
+      <c r="C44" s="71" t="inlineStr">
+        <is>
+          <t>Écart d'au moins 8 %</t>
+        </is>
+      </c>
+      <c r="D44" s="71" t="n"/>
+      <c r="E44" s="71" t="n"/>
+      <c r="F44" s="69" t="n"/>
+      <c r="G44" s="72" t="n"/>
+      <c r="H44" s="72" t="n"/>
+      <c r="I44" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": 0.08}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" outlineLevel="1" ht="15" customHeight="1" s="40">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>exemple</t>
-        </is>
-      </c>
-      <c r="B45" s="75" t="inlineStr">
-        <is>
-          <t>Sites de paris</t>
-        </is>
-      </c>
-      <c r="C45" s="75" t="inlineStr">
-        <is>
-          <t>Ligue 2</t>
-        </is>
-      </c>
-      <c r="D45" s="75" t="inlineStr">
-        <is>
-          <t>fra.2</t>
-        </is>
-      </c>
-      <c r="F45" s="75" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="H45" s="75" t="inlineStr">
-        <is>
-          <t>Ligne d'exemple : ignorée par la tâche</t>
+          <t>cr:seuil:10</t>
+        </is>
+      </c>
+      <c r="B45" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · seuil d'affichage (un seul)</t>
+        </is>
+      </c>
+      <c r="C45" s="71" t="inlineStr">
+        <is>
+          <t>Écart d'au moins 10 %</t>
+        </is>
+      </c>
+      <c r="D45" s="71" t="n"/>
+      <c r="E45" s="71" t="n"/>
+      <c r="F45" s="69" t="n"/>
+      <c r="G45" s="72" t="n"/>
+      <c r="H45" s="72" t="n"/>
+      <c r="I45" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": 0.1}</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="40">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>ajout:1</t>
-        </is>
-      </c>
-      <c r="B46" s="76" t="n"/>
-      <c r="C46" s="76" t="n"/>
-      <c r="D46" s="76" t="n"/>
-      <c r="F46" s="77" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="40">
+          <t>sec:cotes:rapport_ref</t>
+        </is>
+      </c>
+      <c r="B46" s="66" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · comparaison (une seule)</t>
+        </is>
+      </c>
+      <c r="C46" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D46" s="68" t="n"/>
+      <c r="E46" s="68" t="n"/>
+      <c r="F46" s="69" t="n"/>
+      <c r="G46" s="68" t="n"/>
+      <c r="H46" s="68" t="n"/>
+      <c r="I46" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "rapport_ref", "label": "Rapport des écarts · comparaison (une seule)"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" outlineLevel="1" ht="15" customHeight="1" s="40">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>ajout:2</t>
-        </is>
-      </c>
-      <c r="B47" s="76" t="n"/>
-      <c r="C47" s="76" t="n"/>
-      <c r="D47" s="76" t="n"/>
-      <c r="F47" s="77" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="40">
+          <t>cr:ref:moyenne</t>
+        </is>
+      </c>
+      <c r="B47" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · comparaison (une seule)</t>
+        </is>
+      </c>
+      <c r="C47" s="71" t="inlineStr">
+        <is>
+          <t>Moyenne des autres sites</t>
+        </is>
+      </c>
+      <c r="D47" s="71" t="n"/>
+      <c r="E47" s="71" t="inlineStr">
+        <is>
+          <t>la cote du site comparée à la moyenne des autres</t>
+        </is>
+      </c>
+      <c r="F47" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G47" s="72" t="n"/>
+      <c r="H47" s="72" t="n"/>
+      <c r="I47" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": "moyenne"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" outlineLevel="1" ht="15" customHeight="1" s="40">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>ajout:3</t>
-        </is>
-      </c>
-      <c r="B48" s="76" t="n"/>
-      <c r="C48" s="76" t="n"/>
-      <c r="D48" s="76" t="n"/>
-      <c r="F48" s="77" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="40">
-      <c r="A49" s="39" t="inlineStr">
-        <is>
-          <t>ajout:4</t>
-        </is>
-      </c>
-      <c r="B49" s="76" t="n"/>
-      <c r="C49" s="76" t="n"/>
-      <c r="D49" s="76" t="n"/>
-      <c r="F49" s="77" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="40">
-      <c r="A50" s="39" t="inlineStr">
-        <is>
-          <t>ajout:5</t>
-        </is>
-      </c>
-      <c r="B50" s="76" t="n"/>
-      <c r="C50" s="76" t="n"/>
-      <c r="D50" s="76" t="n"/>
-      <c r="F50" s="77" t="n"/>
-    </row>
+          <t>cr:ref:mediane</t>
+        </is>
+      </c>
+      <c r="B48" s="70" t="inlineStr">
+        <is>
+          <t>Rapport des écarts · comparaison (une seule)</t>
+        </is>
+      </c>
+      <c r="C48" s="71" t="inlineStr">
+        <is>
+          <t>Médiane des autres sites</t>
+        </is>
+      </c>
+      <c r="D48" s="71" t="n"/>
+      <c r="E48" s="71" t="inlineStr">
+        <is>
+          <t>moins sensible à un autre site lui-même décalé</t>
+        </is>
+      </c>
+      <c r="F48" s="69" t="n"/>
+      <c r="G48" s="72" t="n"/>
+      <c r="H48" s="72" t="n"/>
+      <c r="I48" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": "mediane"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50"/>
     <row r="51" ht="15" customHeight="1" s="40">
-      <c r="A51" s="39" t="inlineStr">
-        <is>
-          <t>ajout:6</t>
-        </is>
-      </c>
-      <c r="B51" s="76" t="n"/>
-      <c r="C51" s="76" t="n"/>
-      <c r="D51" s="76" t="n"/>
-      <c r="F51" s="77" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="40">
-      <c r="A52" s="39" t="inlineStr">
-        <is>
-          <t>ajout:7</t>
-        </is>
-      </c>
-      <c r="B52" s="76" t="n"/>
-      <c r="C52" s="76" t="n"/>
-      <c r="D52" s="76" t="n"/>
-      <c r="F52" s="77" t="n"/>
+      <c r="B51" s="73" t="inlineStr">
+        <is>
+          <t>MES AJOUTS — tape ce que tu veux ajouter : la tâche essaie de le récupérer et écrit le résultat (✅ / ⚠️ / ❌) dans la colonne « Résultat »</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1" s="40">
+      <c r="B52" s="74" t="inlineStr">
+        <is>
+          <t>Section (Sites de paris ou Compétitions relevées)</t>
+        </is>
+      </c>
+      <c r="C52" s="74" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="D52" s="74" t="inlineStr">
+        <is>
+          <t>Clé The Odds API ou id de compétition du dock</t>
+        </is>
+      </c>
+      <c r="F52" s="74" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G52" s="74" t="inlineStr">
+        <is>
+          <t>Résultat</t>
+        </is>
+      </c>
+      <c r="H52" s="74" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="40">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>ajout:8</t>
-        </is>
-      </c>
-      <c r="B53" s="76" t="n"/>
-      <c r="C53" s="76" t="n"/>
-      <c r="D53" s="76" t="n"/>
-      <c r="F53" s="77" t="n"/>
+          <t>exemple</t>
+        </is>
+      </c>
+      <c r="B53" s="75" t="inlineStr">
+        <is>
+          <t>Sites de paris</t>
+        </is>
+      </c>
+      <c r="C53" s="75" t="inlineStr">
+        <is>
+          <t>Ligue 2</t>
+        </is>
+      </c>
+      <c r="D53" s="75" t="inlineStr">
+        <is>
+          <t>fra.2</t>
+        </is>
+      </c>
+      <c r="F53" s="75" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H53" s="75" t="inlineStr">
+        <is>
+          <t>Ligne d'exemple : ignorée par la tâche</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="40">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>ajout:9</t>
+          <t>ajout:1</t>
         </is>
       </c>
       <c r="B54" s="76" t="n"/>
@@ -6049,7 +6234,7 @@
     <row r="55" ht="15" customHeight="1" s="40">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>ajout:10</t>
+          <t>ajout:2</t>
         </is>
       </c>
       <c r="B55" s="76" t="n"/>
@@ -6060,7 +6245,7 @@
     <row r="56" ht="15" customHeight="1" s="40">
       <c r="A56" s="39" t="inlineStr">
         <is>
-          <t>ajout:11</t>
+          <t>ajout:3</t>
         </is>
       </c>
       <c r="B56" s="76" t="n"/>
@@ -6071,7 +6256,7 @@
     <row r="57" ht="15" customHeight="1" s="40">
       <c r="A57" s="39" t="inlineStr">
         <is>
-          <t>ajout:12</t>
+          <t>ajout:4</t>
         </is>
       </c>
       <c r="B57" s="76" t="n"/>
@@ -6082,7 +6267,7 @@
     <row r="58" ht="15" customHeight="1" s="40">
       <c r="A58" s="39" t="inlineStr">
         <is>
-          <t>ajout:13</t>
+          <t>ajout:5</t>
         </is>
       </c>
       <c r="B58" s="76" t="n"/>
@@ -6093,7 +6278,7 @@
     <row r="59" ht="15" customHeight="1" s="40">
       <c r="A59" s="39" t="inlineStr">
         <is>
-          <t>ajout:14</t>
+          <t>ajout:6</t>
         </is>
       </c>
       <c r="B59" s="76" t="n"/>
@@ -6104,7 +6289,7 @@
     <row r="60" ht="15" customHeight="1" s="40">
       <c r="A60" s="39" t="inlineStr">
         <is>
-          <t>ajout:15</t>
+          <t>ajout:7</t>
         </is>
       </c>
       <c r="B60" s="76" t="n"/>
@@ -6115,7 +6300,7 @@
     <row r="61" ht="15" customHeight="1" s="40">
       <c r="A61" s="39" t="inlineStr">
         <is>
-          <t>ajout:16</t>
+          <t>ajout:8</t>
         </is>
       </c>
       <c r="B61" s="76" t="n"/>
@@ -6126,7 +6311,7 @@
     <row r="62" ht="15" customHeight="1" s="40">
       <c r="A62" s="39" t="inlineStr">
         <is>
-          <t>ajout:17</t>
+          <t>ajout:9</t>
         </is>
       </c>
       <c r="B62" s="76" t="n"/>
@@ -6137,7 +6322,7 @@
     <row r="63" ht="15" customHeight="1" s="40">
       <c r="A63" s="39" t="inlineStr">
         <is>
-          <t>ajout:18</t>
+          <t>ajout:10</t>
         </is>
       </c>
       <c r="B63" s="76" t="n"/>
@@ -6148,7 +6333,7 @@
     <row r="64" ht="15" customHeight="1" s="40">
       <c r="A64" s="39" t="inlineStr">
         <is>
-          <t>ajout:19</t>
+          <t>ajout:11</t>
         </is>
       </c>
       <c r="B64" s="76" t="n"/>
@@ -6159,7 +6344,7 @@
     <row r="65" ht="15" customHeight="1" s="40">
       <c r="A65" s="39" t="inlineStr">
         <is>
-          <t>ajout:20</t>
+          <t>ajout:12</t>
         </is>
       </c>
       <c r="B65" s="76" t="n"/>
@@ -6167,15 +6352,103 @@
       <c r="D65" s="76" t="n"/>
       <c r="F65" s="77" t="n"/>
     </row>
+    <row r="66" ht="15" customHeight="1" s="40">
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>ajout:13</t>
+        </is>
+      </c>
+      <c r="B66" s="76" t="n"/>
+      <c r="C66" s="76" t="n"/>
+      <c r="D66" s="76" t="n"/>
+      <c r="F66" s="77" t="n"/>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="40">
+      <c r="A67" s="39" t="inlineStr">
+        <is>
+          <t>ajout:14</t>
+        </is>
+      </c>
+      <c r="B67" s="76" t="n"/>
+      <c r="C67" s="76" t="n"/>
+      <c r="D67" s="76" t="n"/>
+      <c r="F67" s="77" t="n"/>
+    </row>
+    <row r="68" ht="15" customHeight="1" s="40">
+      <c r="A68" s="39" t="inlineStr">
+        <is>
+          <t>ajout:15</t>
+        </is>
+      </c>
+      <c r="B68" s="76" t="n"/>
+      <c r="C68" s="76" t="n"/>
+      <c r="D68" s="76" t="n"/>
+      <c r="F68" s="77" t="n"/>
+    </row>
+    <row r="69" ht="15" customHeight="1" s="40">
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>ajout:16</t>
+        </is>
+      </c>
+      <c r="B69" s="76" t="n"/>
+      <c r="C69" s="76" t="n"/>
+      <c r="D69" s="76" t="n"/>
+      <c r="F69" s="77" t="n"/>
+    </row>
+    <row r="70" ht="15" customHeight="1" s="40">
+      <c r="A70" s="39" t="inlineStr">
+        <is>
+          <t>ajout:17</t>
+        </is>
+      </c>
+      <c r="B70" s="76" t="n"/>
+      <c r="C70" s="76" t="n"/>
+      <c r="D70" s="76" t="n"/>
+      <c r="F70" s="77" t="n"/>
+    </row>
+    <row r="71" ht="15" customHeight="1" s="40">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>ajout:18</t>
+        </is>
+      </c>
+      <c r="B71" s="76" t="n"/>
+      <c r="C71" s="76" t="n"/>
+      <c r="D71" s="76" t="n"/>
+      <c r="F71" s="77" t="n"/>
+    </row>
+    <row r="72" ht="15" customHeight="1" s="40">
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>ajout:19</t>
+        </is>
+      </c>
+      <c r="B72" s="76" t="n"/>
+      <c r="C72" s="76" t="n"/>
+      <c r="D72" s="76" t="n"/>
+      <c r="F72" s="77" t="n"/>
+    </row>
+    <row r="73" ht="15" customHeight="1" s="40">
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>ajout:20</t>
+        </is>
+      </c>
+      <c r="B73" s="76" t="n"/>
+      <c r="C73" s="76" t="n"/>
+      <c r="D73" s="76" t="n"/>
+      <c r="F73" s="77" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B5:H40"/>
+  <autoFilter ref="B5:H48"/>
   <mergeCells count="4">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B51:H51"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B43:H43"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:H40">
+  <conditionalFormatting sqref="B6:H48">
     <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
       <formula>$F6="Oui"</formula>
     </cfRule>
@@ -6184,7 +6457,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6:F65" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choix" error="Réponds « Oui », « Non » ou laisse vide." type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="F6:F73" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choix" error="Réponds « Oui », « Non » ou laisse vide." type="list" errorStyle="stop" operator="between">
       <formula1>"Oui,Non"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6218,7 +6491,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=accueil;version=1</t>
+          <t>module=accueil;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -7595,6 +7868,2355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:J79"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="1"/>
+  <cols>
+    <col hidden="1" width="14" customWidth="1" style="39" min="1" max="1"/>
+    <col width="26" customWidth="1" style="39" min="2" max="2"/>
+    <col width="22" customWidth="1" style="39" min="3" max="3"/>
+    <col width="34" customWidth="1" style="39" min="4" max="4"/>
+    <col width="40" customWidth="1" style="39" min="5" max="5"/>
+    <col width="30" customWidth="1" style="39" min="6" max="6"/>
+    <col width="8" customWidth="1" style="39" min="7" max="7"/>
+    <col width="26" customWidth="1" style="39" min="8" max="8"/>
+    <col width="34" customWidth="1" style="39" min="9" max="9"/>
+    <col hidden="1" width="10" customWidth="1" style="39" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="40">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>module=applis;version=2</t>
+        </is>
+      </c>
+      <c r="B1" s="61" t="inlineStr">
+        <is>
+          <t>Accueil · applis, dossiers et liens</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="43.5" customHeight="1" s="40">
+      <c r="B2" s="62" t="inlineStr">
+        <is>
+          <t>Chaque appli a 3 liens : iPhone (lien d'ouverture de l'appli), Android (ouvre l'appli ou sa page Google Play) et web (site, utilisé sur PC ou si l'appli manque). Ces liens sont modifiables directement dans le tableau. Aujourd'hui le dock utilise les liens iPhone et web ; les liens Android préparent la version multi-plateforme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="27.75" customHeight="1" s="40">
+      <c r="B3" s="63" t="inlineStr">
+        <is>
+          <t>À remplir : cases jaunes (« Oui » ou « Non »). Ligne « ▸ toute la section » = tous ses éléments, sauf ceux marqués « Non ». Un seul élément coché suffit pour que sa section apparaisse. Colonne « Résultat » : remplie par la tâche GitHub après dépôt du classeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="21.75" customHeight="1" s="40">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="inlineStr">
+        <is>
+          <t>Appli</t>
+        </is>
+      </c>
+      <c r="D5" s="64" t="inlineStr">
+        <is>
+          <t>Lien iPhone</t>
+        </is>
+      </c>
+      <c r="E5" s="64" t="inlineStr">
+        <is>
+          <t>Lien Android</t>
+        </is>
+      </c>
+      <c r="F5" s="64" t="inlineStr">
+        <is>
+          <t>Lien web</t>
+        </is>
+      </c>
+      <c r="G5" s="65" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H5" s="64" t="inlineStr">
+        <is>
+          <t>Résultat</t>
+        </is>
+      </c>
+      <c r="I5" s="64" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="J5" s="64" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="40">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:accueil</t>
+        </is>
+      </c>
+      <c r="B6" s="66" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D6" s="68" t="n"/>
+      <c r="E6" s="68" t="n"/>
+      <c r="F6" s="68" t="n"/>
+      <c r="G6" s="69" t="n"/>
+      <c r="H6" s="68" t="n"/>
+      <c r="I6" s="68" t="n"/>
+      <c r="J6" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "accueil", "label": "Écran d'accueil", "type": "liste"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:finance</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C7" s="71" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D7" s="71" t="inlineStr">
+        <is>
+          <t>dossier finance</t>
+        </is>
+      </c>
+      <c r="E7" s="71" t="n"/>
+      <c r="F7" s="71" t="n"/>
+      <c r="G7" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="n"/>
+      <c r="I7" s="72" t="n"/>
+      <c r="J7" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Finance", "type": "folder", "target": "finance"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A8" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:travail</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C8" s="71" t="inlineStr">
+        <is>
+          <t>Travail</t>
+        </is>
+      </c>
+      <c r="D8" s="71" t="inlineStr">
+        <is>
+          <t>dossier travail</t>
+        </is>
+      </c>
+      <c r="E8" s="71" t="n"/>
+      <c r="F8" s="71" t="n"/>
+      <c r="G8" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="72" t="n"/>
+      <c r="J8" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Travail", "type": "folder", "target": "travail"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:medias</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C9" s="71" t="inlineStr">
+        <is>
+          <t>Médias</t>
+        </is>
+      </c>
+      <c r="D9" s="71" t="inlineStr">
+        <is>
+          <t>dossier medias</t>
+        </is>
+      </c>
+      <c r="E9" s="71" t="n"/>
+      <c r="F9" s="71" t="n"/>
+      <c r="G9" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H9" s="72" t="n"/>
+      <c r="I9" s="72" t="n"/>
+      <c r="J9" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Médias", "type": "folder", "target": "medias"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:jeux</t>
+        </is>
+      </c>
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C10" s="71" t="inlineStr">
+        <is>
+          <t>Jeux</t>
+        </is>
+      </c>
+      <c r="D10" s="71" t="inlineStr">
+        <is>
+          <t>dossier jeux</t>
+        </is>
+      </c>
+      <c r="E10" s="71" t="n"/>
+      <c r="F10" s="71" t="n"/>
+      <c r="G10" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H10" s="72" t="n"/>
+      <c r="I10" s="72" t="n"/>
+      <c r="J10" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Jeux", "type": "folder", "target": "jeux"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:videos</t>
+        </is>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C11" s="71" t="inlineStr">
+        <is>
+          <t>Vidéos</t>
+        </is>
+      </c>
+      <c r="D11" s="71" t="inlineStr">
+        <is>
+          <t>page videos.html</t>
+        </is>
+      </c>
+      <c r="E11" s="71" t="n"/>
+      <c r="F11" s="71" t="n"/>
+      <c r="G11" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H11" s="72" t="n"/>
+      <c r="I11" s="72" t="n"/>
+      <c r="J11" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Vidéos", "type": "page", "url": "videos.html", "icon": "play", "color": "--t-brick"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>ap:accueil:sports</t>
+        </is>
+      </c>
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C12" s="71" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="D12" s="71" t="inlineStr">
+        <is>
+          <t>page sport.html</t>
+        </is>
+      </c>
+      <c r="E12" s="71" t="n"/>
+      <c r="F12" s="71" t="n"/>
+      <c r="G12" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H12" s="72" t="n"/>
+      <c r="I12" s="72" t="n"/>
+      <c r="J12" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Sports", "type": "page", "url": "sport.html", "live": true, "color": "--t-plum"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="40">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:dossier-finance</t>
+        </is>
+      </c>
+      <c r="B13" s="66" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C13" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D13" s="68" t="n"/>
+      <c r="E13" s="68" t="n"/>
+      <c r="F13" s="68" t="n"/>
+      <c r="G13" s="69" t="n"/>
+      <c r="H13" s="68" t="n"/>
+      <c r="I13" s="68" t="n"/>
+      <c r="J13" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "finance", "label": "Finance", "type": "dossier"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>ap:finance:trade-republic</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C14" s="71" t="inlineStr">
+        <is>
+          <t>Trade Republic</t>
+        </is>
+      </c>
+      <c r="D14" s="71" t="inlineStr">
+        <is>
+          <t>traderepublic://</t>
+        </is>
+      </c>
+      <c r="E14" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=de.traderepublic.app;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dde.traderepublic.app;end</t>
+        </is>
+      </c>
+      <c r="F14" s="71" t="inlineStr">
+        <is>
+          <t>https://app.traderepublic.com</t>
+        </is>
+      </c>
+      <c r="G14" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H14" s="72" t="n"/>
+      <c r="I14" s="72" t="n"/>
+      <c r="J14" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Trade Republic", "mono": "TR", "color": "--t-char", "store": "Trade Republic", "app": "traderepublic://", "web": "https://app.traderepublic.com", "android": "intent://#Intent;package=de.traderepublic.app;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dde.traderepublic.app;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>ap:finance:boursobank</t>
+        </is>
+      </c>
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C15" s="71" t="inlineStr">
+        <is>
+          <t>BoursoBank</t>
+        </is>
+      </c>
+      <c r="D15" s="71" t="inlineStr">
+        <is>
+          <t>shortcuts://run-shortcut?name=BoursoBank</t>
+        </is>
+      </c>
+      <c r="E15" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.boursorama.android.clients;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.boursorama.android.clients;end</t>
+        </is>
+      </c>
+      <c r="F15" s="71" t="n"/>
+      <c r="G15" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H15" s="72" t="n"/>
+      <c r="I15" s="72" t="n"/>
+      <c r="J15" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "BoursoBank", "mono": "Bo", "color": "--t-rose", "store": "BoursoBank", "app": "shortcuts://run-shortcut?name=BoursoBank", "android": "intent://#Intent;package=com.boursorama.android.clients;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.boursorama.android.clients;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>ap:finance:cyberplus</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C16" s="71" t="inlineStr">
+        <is>
+          <t>Cyberplus</t>
+        </is>
+      </c>
+      <c r="D16" s="71" t="inlineStr">
+        <is>
+          <t>cyberplus://</t>
+        </is>
+      </c>
+      <c r="E16" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=fr.banquepopulaire.cyberplus;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dfr.banquepopulaire.cyberplus;end</t>
+        </is>
+      </c>
+      <c r="F16" s="71" t="inlineStr">
+        <is>
+          <t>https://www.banquepopulaire.fr</t>
+        </is>
+      </c>
+      <c r="G16" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H16" s="72" t="n"/>
+      <c r="I16" s="72" t="n"/>
+      <c r="J16" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Cyberplus", "mono": "BP", "color": "--t-brick", "store": "Banque Populaire", "app": "cyberplus://", "web": "https://www.banquepopulaire.fr", "android": "intent://#Intent;package=fr.banquepopulaire.cyberplus;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dfr.banquepopulaire.cyberplus;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>ap:finance:swile</t>
+        </is>
+      </c>
+      <c r="B17" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="inlineStr">
+        <is>
+          <t>Swile</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="inlineStr">
+        <is>
+          <t>swile://</t>
+        </is>
+      </c>
+      <c r="E17" s="71" t="n"/>
+      <c r="F17" s="71" t="inlineStr">
+        <is>
+          <t>https://app.swile.co</t>
+        </is>
+      </c>
+      <c r="G17" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H17" s="72" t="n"/>
+      <c r="I17" s="72" t="inlineStr">
+        <is>
+          <t>identifiant Android à compléter</t>
+        </is>
+      </c>
+      <c r="J17" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Swile", "mono": "Sw", "color": "--t-plum", "store": "Swile", "app": "swile://", "web": "https://app.swile.co"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>ap:finance:esalia</t>
+        </is>
+      </c>
+      <c r="B18" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Finance</t>
+        </is>
+      </c>
+      <c r="C18" s="71" t="inlineStr">
+        <is>
+          <t>Esalia</t>
+        </is>
+      </c>
+      <c r="D18" s="71" t="inlineStr">
+        <is>
+          <t>shortcuts://run-shortcut?name=Esalia</t>
+        </is>
+      </c>
+      <c r="E18" s="71" t="n"/>
+      <c r="F18" s="71" t="n"/>
+      <c r="G18" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H18" s="72" t="n"/>
+      <c r="I18" s="72" t="inlineStr">
+        <is>
+          <t>identifiant Android à compléter</t>
+        </is>
+      </c>
+      <c r="J18" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Esalia", "mono": "Es", "color": "--t-teal", "store": "Esalia", "app": "shortcuts://run-shortcut?name=Esalia"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="40">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:dossier-medias</t>
+        </is>
+      </c>
+      <c r="B19" s="66" t="inlineStr">
+        <is>
+          <t>Dossier Médias</t>
+        </is>
+      </c>
+      <c r="C19" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D19" s="68" t="n"/>
+      <c r="E19" s="68" t="n"/>
+      <c r="F19" s="68" t="n"/>
+      <c r="G19" s="69" t="n"/>
+      <c r="H19" s="68" t="n"/>
+      <c r="I19" s="68" t="n"/>
+      <c r="J19" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "medias", "label": "Médias", "type": "dossier"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>ap:medias:videolite</t>
+        </is>
+      </c>
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Médias</t>
+        </is>
+      </c>
+      <c r="C20" s="71" t="inlineStr">
+        <is>
+          <t>VideoLite</t>
+        </is>
+      </c>
+      <c r="D20" s="71" t="inlineStr">
+        <is>
+          <t>videolite://</t>
+        </is>
+      </c>
+      <c r="E20" s="71" t="n"/>
+      <c r="F20" s="71" t="n"/>
+      <c r="G20" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H20" s="72" t="n"/>
+      <c r="I20" s="72" t="inlineStr">
+        <is>
+          <t>appli iPhone uniquement ?</t>
+        </is>
+      </c>
+      <c r="J20" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "VideoLite", "mono": "VL", "color": "--t-plum", "store": "VideoLite", "app": "videolite://", "alt": "VideoLite"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>ap:medias:canal</t>
+        </is>
+      </c>
+      <c r="B21" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Médias</t>
+        </is>
+      </c>
+      <c r="C21" s="71" t="inlineStr">
+        <is>
+          <t>Canal+</t>
+        </is>
+      </c>
+      <c r="D21" s="71" t="inlineStr">
+        <is>
+          <t>mycanal://</t>
+        </is>
+      </c>
+      <c r="E21" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.canal.android.canal;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.canal.android.canal;end</t>
+        </is>
+      </c>
+      <c r="F21" s="71" t="inlineStr">
+        <is>
+          <t>https://www.canalplus.com</t>
+        </is>
+      </c>
+      <c r="G21" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H21" s="72" t="n"/>
+      <c r="I21" s="72" t="n"/>
+      <c r="J21" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Canal+", "mono": "C+", "color": "--t-char", "store": "CANAL+", "app": "mycanal://", "alt": "CANAL+", "web": "https://www.canalplus.com", "android": "intent://#Intent;package=com.canal.android.canal;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.canal.android.canal;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>ap:medias:prime-video</t>
+        </is>
+      </c>
+      <c r="B22" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Médias</t>
+        </is>
+      </c>
+      <c r="C22" s="71" t="inlineStr">
+        <is>
+          <t>Prime Video</t>
+        </is>
+      </c>
+      <c r="D22" s="71" t="inlineStr">
+        <is>
+          <t>aiv://</t>
+        </is>
+      </c>
+      <c r="E22" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.amazon.avod.thirdpartyclient;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.amazon.avod.thirdpartyclient;end</t>
+        </is>
+      </c>
+      <c r="F22" s="71" t="inlineStr">
+        <is>
+          <t>https://www.primevideo.com</t>
+        </is>
+      </c>
+      <c r="G22" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H22" s="72" t="n"/>
+      <c r="I22" s="72" t="n"/>
+      <c r="J22" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Prime Video", "mono": "PV", "color": "--t-slate", "store": "Amazon Prime Video", "app": "aiv://", "web": "https://www.primevideo.com", "android": "intent://#Intent;package=com.amazon.avod.thirdpartyclient;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.amazon.avod.thirdpartyclient;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>ap:medias:smartersplayerlite</t>
+        </is>
+      </c>
+      <c r="B23" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Médias</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="inlineStr">
+        <is>
+          <t>SmartersPlayerLite</t>
+        </is>
+      </c>
+      <c r="D23" s="71" t="inlineStr">
+        <is>
+          <t>smartersplayerlite://</t>
+        </is>
+      </c>
+      <c r="E23" s="71" t="n"/>
+      <c r="F23" s="71" t="n"/>
+      <c r="G23" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H23" s="72" t="n"/>
+      <c r="I23" s="72" t="inlineStr">
+        <is>
+          <t>identifiant Android à compléter</t>
+        </is>
+      </c>
+      <c r="J23" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "SmartersPlayerLite", "mono": "SP", "color": "--t-teal", "store": "Smarters Player Lite", "app": "smartersplayerlite://", "alt": "SmartersPlayerLite"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="40">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:dossier-jeux</t>
+        </is>
+      </c>
+      <c r="B24" s="66" t="inlineStr">
+        <is>
+          <t>Dossier Jeux</t>
+        </is>
+      </c>
+      <c r="C24" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D24" s="68" t="n"/>
+      <c r="E24" s="68" t="n"/>
+      <c r="F24" s="68" t="n"/>
+      <c r="G24" s="69" t="n"/>
+      <c r="H24" s="68" t="n"/>
+      <c r="I24" s="68" t="n"/>
+      <c r="J24" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "jeux", "label": "Jeux", "type": "dossier"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>ap:jeux:chess</t>
+        </is>
+      </c>
+      <c r="B25" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Jeux</t>
+        </is>
+      </c>
+      <c r="C25" s="71" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="D25" s="71" t="inlineStr">
+        <is>
+          <t>shortcuts://run-shortcut?name=Chess</t>
+        </is>
+      </c>
+      <c r="E25" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.chess;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.chess;end</t>
+        </is>
+      </c>
+      <c r="F25" s="71" t="n"/>
+      <c r="G25" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H25" s="72" t="n"/>
+      <c r="I25" s="72" t="n"/>
+      <c r="J25" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Chess", "mono": "♞", "color": "--t-olive", "store": "Chess Play and Learn", "app": "shortcuts://run-shortcut?name=Chess", "android": "intent://#Intent;package=com.chess;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.chess;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A26" s="39" t="inlineStr">
+        <is>
+          <t>ap:jeux:brawl-stars</t>
+        </is>
+      </c>
+      <c r="B26" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Jeux</t>
+        </is>
+      </c>
+      <c r="C26" s="71" t="inlineStr">
+        <is>
+          <t>Brawl Stars</t>
+        </is>
+      </c>
+      <c r="D26" s="71" t="inlineStr">
+        <is>
+          <t>brawlstars://</t>
+        </is>
+      </c>
+      <c r="E26" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.supercell.brawlstars;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.supercell.brawlstars;end</t>
+        </is>
+      </c>
+      <c r="F26" s="71" t="n"/>
+      <c r="G26" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H26" s="72" t="n"/>
+      <c r="I26" s="72" t="n"/>
+      <c r="J26" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Brawl Stars", "mono": "BS", "color": "--t-ochre", "store": "Brawl Stars", "app": "brawlstars://", "android": "intent://#Intent;package=com.supercell.brawlstars;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.supercell.brawlstars;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>ap:jeux:songs-of-conquest</t>
+        </is>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Jeux</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>Songs of Conquest</t>
+        </is>
+      </c>
+      <c r="D27" s="71" t="inlineStr">
+        <is>
+          <t>shortcuts://run-shortcut?name=Songs%20of%20Conquest</t>
+        </is>
+      </c>
+      <c r="E27" s="71" t="n"/>
+      <c r="F27" s="71" t="n"/>
+      <c r="G27" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H27" s="72" t="n"/>
+      <c r="I27" s="72" t="inlineStr">
+        <is>
+          <t>version mobile à vérifier</t>
+        </is>
+      </c>
+      <c r="J27" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Songs of Conquest", "mono": "SC", "color": "--t-plum", "store": "Songs of Conquest", "app": "shortcuts://run-shortcut?name=Songs%20of%20Conquest"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="40">
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:dossier-travail</t>
+        </is>
+      </c>
+      <c r="B28" s="66" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D28" s="68" t="n"/>
+      <c r="E28" s="68" t="n"/>
+      <c r="F28" s="68" t="n"/>
+      <c r="G28" s="69" t="n"/>
+      <c r="H28" s="68" t="n"/>
+      <c r="I28" s="68" t="n"/>
+      <c r="J28" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "travail", "label": "Travail", "type": "dossier"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:outlook</t>
+        </is>
+      </c>
+      <c r="B29" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="D29" s="71" t="inlineStr">
+        <is>
+          <t>ms-outlook://</t>
+        </is>
+      </c>
+      <c r="E29" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.office.outlook;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.outlook;end</t>
+        </is>
+      </c>
+      <c r="F29" s="71" t="inlineStr">
+        <is>
+          <t>https://outlook.office.com</t>
+        </is>
+      </c>
+      <c r="G29" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H29" s="72" t="n"/>
+      <c r="I29" s="72" t="n"/>
+      <c r="J29" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Outlook", "mono": "O", "color": "--t-slate", "store": "Microsoft Outlook", "app": "ms-outlook://", "web": "https://outlook.office.com", "android": "intent://#Intent;package=com.microsoft.office.outlook;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.outlook;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:teams</t>
+        </is>
+      </c>
+      <c r="B30" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C30" s="71" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="D30" s="71" t="inlineStr">
+        <is>
+          <t>msteams://</t>
+        </is>
+      </c>
+      <c r="E30" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.teams;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.teams;end</t>
+        </is>
+      </c>
+      <c r="F30" s="71" t="inlineStr">
+        <is>
+          <t>https://teams.microsoft.com</t>
+        </is>
+      </c>
+      <c r="G30" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H30" s="72" t="n"/>
+      <c r="I30" s="72" t="n"/>
+      <c r="J30" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Teams", "mono": "T", "color": "--t-plum", "store": "Microsoft Teams", "app": "msteams://", "web": "https://teams.microsoft.com", "android": "intent://#Intent;package=com.microsoft.teams;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.teams;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:word</t>
+        </is>
+      </c>
+      <c r="B31" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C31" s="71" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D31" s="71" t="inlineStr">
+        <is>
+          <t>ms-word://</t>
+        </is>
+      </c>
+      <c r="E31" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.office.word;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.word;end</t>
+        </is>
+      </c>
+      <c r="F31" s="71" t="inlineStr">
+        <is>
+          <t>https://www.office.com</t>
+        </is>
+      </c>
+      <c r="G31" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H31" s="72" t="n"/>
+      <c r="I31" s="72" t="n"/>
+      <c r="J31" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Word", "mono": "W", "color": "--t-brick", "store": "Microsoft Word", "app": "ms-word://", "web": "https://www.office.com", "android": "intent://#Intent;package=com.microsoft.office.word;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.word;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:powerpoint</t>
+        </is>
+      </c>
+      <c r="B32" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C32" s="71" t="inlineStr">
+        <is>
+          <t>PowerPoint</t>
+        </is>
+      </c>
+      <c r="D32" s="71" t="inlineStr">
+        <is>
+          <t>ms-powerpoint://</t>
+        </is>
+      </c>
+      <c r="E32" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.office.powerpoint;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.powerpoint;end</t>
+        </is>
+      </c>
+      <c r="F32" s="71" t="inlineStr">
+        <is>
+          <t>https://www.office.com</t>
+        </is>
+      </c>
+      <c r="G32" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H32" s="72" t="n"/>
+      <c r="I32" s="72" t="n"/>
+      <c r="J32" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "PowerPoint", "mono": "P", "color": "--t-rose", "store": "Microsoft PowerPoint", "app": "ms-powerpoint://", "web": "https://www.office.com", "android": "intent://#Intent;package=com.microsoft.office.powerpoint;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.powerpoint;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:onenote</t>
+        </is>
+      </c>
+      <c r="B33" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C33" s="71" t="inlineStr">
+        <is>
+          <t>OneNote</t>
+        </is>
+      </c>
+      <c r="D33" s="71" t="inlineStr">
+        <is>
+          <t>onenote://</t>
+        </is>
+      </c>
+      <c r="E33" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.office.onenote;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.onenote;end</t>
+        </is>
+      </c>
+      <c r="F33" s="71" t="inlineStr">
+        <is>
+          <t>https://www.onenote.com</t>
+        </is>
+      </c>
+      <c r="G33" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H33" s="72" t="n"/>
+      <c r="I33" s="72" t="n"/>
+      <c r="J33" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "OneNote", "mono": "N", "color": "--t-plum", "store": "Microsoft OneNote", "app": "onenote://", "web": "https://www.onenote.com", "android": "intent://#Intent;package=com.microsoft.office.onenote;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.office.onenote;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A34" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:power-bi</t>
+        </is>
+      </c>
+      <c r="B34" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C34" s="71" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="D34" s="71" t="inlineStr">
+        <is>
+          <t>mspbi://</t>
+        </is>
+      </c>
+      <c r="E34" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.powerbim;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.powerbim;end</t>
+        </is>
+      </c>
+      <c r="F34" s="71" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com</t>
+        </is>
+      </c>
+      <c r="G34" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H34" s="72" t="n"/>
+      <c r="I34" s="72" t="n"/>
+      <c r="J34" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Power BI", "mono": "BI", "color": "--t-ochre", "store": "Microsoft Power BI", "app": "mspbi://", "web": "https://app.powerbi.com", "android": "intent://#Intent;package=com.microsoft.powerbim;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.powerbim;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A35" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:sap-concur</t>
+        </is>
+      </c>
+      <c r="B35" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C35" s="71" t="inlineStr">
+        <is>
+          <t>SAP Concur</t>
+        </is>
+      </c>
+      <c r="D35" s="71" t="inlineStr">
+        <is>
+          <t>shortcuts://run-shortcut?name=SAP%20Concur</t>
+        </is>
+      </c>
+      <c r="E35" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.concur.breeze;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.concur.breeze;end</t>
+        </is>
+      </c>
+      <c r="F35" s="71" t="n"/>
+      <c r="G35" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H35" s="72" t="n"/>
+      <c r="I35" s="72" t="n"/>
+      <c r="J35" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "SAP Concur", "mono": "Cc", "color": "--t-teal", "store": "SAP Concur", "app": "shortcuts://run-shortcut?name=SAP%20Concur", "android": "intent://#Intent;package=com.concur.breeze;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.concur.breeze;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:fichiers</t>
+        </is>
+      </c>
+      <c r="B36" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C36" s="71" t="inlineStr">
+        <is>
+          <t>Fichiers</t>
+        </is>
+      </c>
+      <c r="D36" s="71" t="inlineStr">
+        <is>
+          <t>shareddocuments://</t>
+        </is>
+      </c>
+      <c r="E36" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.google.android.apps.nbu.files;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.nbu.files;end</t>
+        </is>
+      </c>
+      <c r="F36" s="71" t="n"/>
+      <c r="G36" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H36" s="72" t="n"/>
+      <c r="I36" s="72" t="inlineStr">
+        <is>
+          <t>équivalent Android : Files by Google</t>
+        </is>
+      </c>
+      <c r="J36" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Fichiers", "icon": "folder", "color": "--t-slate", "storeId": "1232058109", "app": "shareddocuments://", "android": "intent://#Intent;package=com.google.android.apps.nbu.files;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.nbu.files;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:proton-drive</t>
+        </is>
+      </c>
+      <c r="B37" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C37" s="71" t="inlineStr">
+        <is>
+          <t>Proton Drive</t>
+        </is>
+      </c>
+      <c r="D37" s="71" t="inlineStr">
+        <is>
+          <t>protondrive://</t>
+        </is>
+      </c>
+      <c r="E37" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=me.proton.android.drive;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dme.proton.android.drive;end</t>
+        </is>
+      </c>
+      <c r="F37" s="71" t="inlineStr">
+        <is>
+          <t>https://drive.proton.me</t>
+        </is>
+      </c>
+      <c r="G37" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H37" s="72" t="n"/>
+      <c r="I37" s="72" t="n"/>
+      <c r="J37" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Proton Drive", "mono": "PD", "color": "--t-char", "store": "Proton Drive", "app": "protondrive://", "web": "https://drive.proton.me", "android": "intent://#Intent;package=me.proton.android.drive;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dme.proton.android.drive;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A38" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:portail-entreprise</t>
+        </is>
+      </c>
+      <c r="B38" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C38" s="71" t="inlineStr">
+        <is>
+          <t>Portail Entreprise</t>
+        </is>
+      </c>
+      <c r="D38" s="71" t="inlineStr">
+        <is>
+          <t>companyportal://</t>
+        </is>
+      </c>
+      <c r="E38" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.microsoft.windowsintune.companyportal;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.windowsintune.companyportal;end</t>
+        </is>
+      </c>
+      <c r="F38" s="71" t="n"/>
+      <c r="G38" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H38" s="72" t="n"/>
+      <c r="I38" s="72" t="n"/>
+      <c r="J38" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Portail Entreprise", "mono": "PE", "color": "--t-slate", "store": "Intune Company Portal", "app": "companyportal://", "android": "intent://#Intent;package=com.microsoft.windowsintune.companyportal;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.microsoft.windowsintune.companyportal;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:authenticator</t>
+        </is>
+      </c>
+      <c r="B39" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C39" s="71" t="inlineStr">
+        <is>
+          <t>Authenticator</t>
+        </is>
+      </c>
+      <c r="D39" s="71" t="inlineStr">
+        <is>
+          <t>msauth://</t>
+        </is>
+      </c>
+      <c r="E39" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.azure.authenticator;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.azure.authenticator;end</t>
+        </is>
+      </c>
+      <c r="F39" s="71" t="n"/>
+      <c r="G39" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H39" s="72" t="n"/>
+      <c r="I39" s="72" t="n"/>
+      <c r="J39" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Authenticator", "mono": "Au", "color": "--t-olive", "store": "Microsoft Authenticator", "app": "msauth://", "android": "intent://#Intent;package=com.azure.authenticator;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.azure.authenticator;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A40" s="39" t="inlineStr">
+        <is>
+          <t>ap:travail:linkedin</t>
+        </is>
+      </c>
+      <c r="B40" s="70" t="inlineStr">
+        <is>
+          <t>Dossier Travail</t>
+        </is>
+      </c>
+      <c r="C40" s="71" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="D40" s="71" t="inlineStr">
+        <is>
+          <t>linkedin://</t>
+        </is>
+      </c>
+      <c r="E40" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.linkedin.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.linkedin.android;end</t>
+        </is>
+      </c>
+      <c r="F40" s="71" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com</t>
+        </is>
+      </c>
+      <c r="G40" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H40" s="72" t="n"/>
+      <c r="I40" s="72" t="n"/>
+      <c r="J40" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "LinkedIn", "mono": "in", "color": "--t-slate", "store": "LinkedIn", "app": "linkedin://", "web": "https://www.linkedin.com", "android": "intent://#Intent;package=com.linkedin.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.linkedin.android;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="40">
+      <c r="A41" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:bas_gauche</t>
+        </is>
+      </c>
+      <c r="B41" s="66" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · gauche</t>
+        </is>
+      </c>
+      <c r="C41" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D41" s="68" t="n"/>
+      <c r="E41" s="68" t="n"/>
+      <c r="F41" s="68" t="n"/>
+      <c r="G41" s="69" t="n"/>
+      <c r="H41" s="68" t="n"/>
+      <c r="I41" s="68" t="n"/>
+      <c r="J41" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "bas_gauche", "label": "Bandeau du bas · gauche", "type": "liste"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A42" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_gauche:claude</t>
+        </is>
+      </c>
+      <c r="B42" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · gauche</t>
+        </is>
+      </c>
+      <c r="C42" s="71" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D42" s="71" t="inlineStr">
+        <is>
+          <t>claude://</t>
+        </is>
+      </c>
+      <c r="E42" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.anthropic.claude;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.anthropic.claude;end</t>
+        </is>
+      </c>
+      <c r="F42" s="71" t="inlineStr">
+        <is>
+          <t>https://claude.ai</t>
+        </is>
+      </c>
+      <c r="G42" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H42" s="72" t="n"/>
+      <c r="I42" s="72" t="n"/>
+      <c r="J42" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Claude", "icon": "spark", "app": "claude://", "alt": "Claude", "web": "https://claude.ai", "android": "intent://#Intent;package=com.anthropic.claude;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.anthropic.claude;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A43" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_gauche:whatsapp</t>
+        </is>
+      </c>
+      <c r="B43" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · gauche</t>
+        </is>
+      </c>
+      <c r="C43" s="71" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D43" s="71" t="inlineStr">
+        <is>
+          <t>whatsapp://</t>
+        </is>
+      </c>
+      <c r="E43" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.whatsapp;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.whatsapp;end</t>
+        </is>
+      </c>
+      <c r="F43" s="71" t="inlineStr">
+        <is>
+          <t>https://web.whatsapp.com</t>
+        </is>
+      </c>
+      <c r="G43" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H43" s="72" t="n"/>
+      <c r="I43" s="72" t="n"/>
+      <c r="J43" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "WhatsApp", "icon": "round", "app": "whatsapp://", "web": "https://web.whatsapp.com", "android": "intent://#Intent;package=com.whatsapp;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.whatsapp;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_gauche:messenger</t>
+        </is>
+      </c>
+      <c r="B44" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · gauche</t>
+        </is>
+      </c>
+      <c r="C44" s="71" t="inlineStr">
+        <is>
+          <t>Messenger</t>
+        </is>
+      </c>
+      <c r="D44" s="71" t="inlineStr">
+        <is>
+          <t>fb-messenger://</t>
+        </is>
+      </c>
+      <c r="E44" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.facebook.orca;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.facebook.orca;end</t>
+        </is>
+      </c>
+      <c r="F44" s="71" t="inlineStr">
+        <is>
+          <t>https://www.messenger.com</t>
+        </is>
+      </c>
+      <c r="G44" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H44" s="72" t="n"/>
+      <c r="I44" s="72" t="n"/>
+      <c r="J44" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Messenger", "icon": "duo", "app": "fb-messenger://", "web": "https://www.messenger.com", "android": "intent://#Intent;package=com.facebook.orca;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.facebook.orca;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A45" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_gauche:x</t>
+        </is>
+      </c>
+      <c r="B45" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · gauche</t>
+        </is>
+      </c>
+      <c r="C45" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D45" s="71" t="inlineStr">
+        <is>
+          <t>twitter://</t>
+        </is>
+      </c>
+      <c r="E45" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.twitter.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.twitter.android;end</t>
+        </is>
+      </c>
+      <c r="F45" s="71" t="inlineStr">
+        <is>
+          <t>https://x.com</t>
+        </is>
+      </c>
+      <c r="G45" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H45" s="72" t="n"/>
+      <c r="I45" s="72" t="n"/>
+      <c r="J45" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "X", "icon": "xmark", "app": "twitter://", "web": "https://x.com", "android": "intent://#Intent;package=com.twitter.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.twitter.android;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15" customHeight="1" s="40">
+      <c r="A46" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:bas_droite</t>
+        </is>
+      </c>
+      <c r="B46" s="66" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · droite</t>
+        </is>
+      </c>
+      <c r="C46" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D46" s="68" t="n"/>
+      <c r="E46" s="68" t="n"/>
+      <c r="F46" s="68" t="n"/>
+      <c r="G46" s="69" t="n"/>
+      <c r="H46" s="68" t="n"/>
+      <c r="I46" s="68" t="n"/>
+      <c r="J46" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "bas_droite", "label": "Bandeau du bas · droite", "type": "liste"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A47" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_droite:proton-vpn</t>
+        </is>
+      </c>
+      <c r="B47" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · droite</t>
+        </is>
+      </c>
+      <c r="C47" s="71" t="inlineStr">
+        <is>
+          <t>Proton VPN</t>
+        </is>
+      </c>
+      <c r="D47" s="71" t="inlineStr">
+        <is>
+          <t>protonvpn://</t>
+        </is>
+      </c>
+      <c r="E47" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=ch.protonvpn.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dch.protonvpn.android;end</t>
+        </is>
+      </c>
+      <c r="F47" s="71" t="n"/>
+      <c r="G47" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H47" s="72" t="n"/>
+      <c r="I47" s="72" t="n"/>
+      <c r="J47" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Proton VPN", "icon": "network", "app": "protonvpn://", "alt": "Proton VPN", "android": "intent://#Intent;package=ch.protonvpn.android;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dch.protonvpn.android;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A48" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_droite:bitwarden</t>
+        </is>
+      </c>
+      <c r="B48" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · droite</t>
+        </is>
+      </c>
+      <c r="C48" s="71" t="inlineStr">
+        <is>
+          <t>Bitwarden</t>
+        </is>
+      </c>
+      <c r="D48" s="71" t="inlineStr">
+        <is>
+          <t>bitwarden://</t>
+        </is>
+      </c>
+      <c r="E48" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.x8bit.bitwarden;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.x8bit.bitwarden;end</t>
+        </is>
+      </c>
+      <c r="F48" s="71" t="inlineStr">
+        <is>
+          <t>https://vault.bitwarden.eu</t>
+        </is>
+      </c>
+      <c r="G48" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H48" s="72" t="n"/>
+      <c r="I48" s="72" t="n"/>
+      <c r="J48" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Bitwarden", "icon": "shield", "app": "bitwarden://", "alt": "Bitwarden", "web": "https://vault.bitwarden.eu", "android": "intent://#Intent;package=com.x8bit.bitwarden;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.x8bit.bitwarden;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A49" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_droite:cartes</t>
+        </is>
+      </c>
+      <c r="B49" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · droite</t>
+        </is>
+      </c>
+      <c r="C49" s="71" t="inlineStr">
+        <is>
+          <t>Cartes</t>
+        </is>
+      </c>
+      <c r="D49" s="71" t="inlineStr">
+        <is>
+          <t>shoebox://</t>
+        </is>
+      </c>
+      <c r="E49" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.google.android.apps.walletnfcrel;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.walletnfcrel;end</t>
+        </is>
+      </c>
+      <c r="F49" s="71" t="n"/>
+      <c r="G49" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H49" s="72" t="n"/>
+      <c r="I49" s="72" t="inlineStr">
+        <is>
+          <t>équivalent Android : Google Wallet</t>
+        </is>
+      </c>
+      <c r="J49" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Cartes", "icon": "card", "app": "shoebox://", "android": "intent://#Intent;package=com.google.android.apps.walletnfcrel;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.walletnfcrel;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A50" s="39" t="inlineStr">
+        <is>
+          <t>ap:bas_droite:navigation</t>
+        </is>
+      </c>
+      <c r="B50" s="70" t="inlineStr">
+        <is>
+          <t>Bandeau du bas · droite</t>
+        </is>
+      </c>
+      <c r="C50" s="71" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="D50" s="71" t="inlineStr">
+        <is>
+          <t>choix de l'appli de navigation</t>
+        </is>
+      </c>
+      <c r="E50" s="71" t="n"/>
+      <c r="F50" s="71" t="n"/>
+      <c r="G50" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H50" s="72" t="n"/>
+      <c r="I50" s="72" t="n"/>
+      <c r="J50" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Navigation", "icon": "nav", "action": "nav"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="40">
+      <c r="A51" s="39" t="inlineStr">
+        <is>
+          <t>sec:applis:navigation</t>
+        </is>
+      </c>
+      <c r="B51" s="66" t="inlineStr">
+        <is>
+          <t>Applis proposées par Navigation</t>
+        </is>
+      </c>
+      <c r="C51" s="67" t="inlineStr">
+        <is>
+          <t>▸ toute la section</t>
+        </is>
+      </c>
+      <c r="D51" s="68" t="n"/>
+      <c r="E51" s="68" t="n"/>
+      <c r="F51" s="68" t="n"/>
+      <c r="G51" s="69" t="n"/>
+      <c r="H51" s="68" t="n"/>
+      <c r="I51" s="68" t="n"/>
+      <c r="J51" s="39" t="inlineStr">
+        <is>
+          <t>{"id": "navigation", "label": "Applis proposées par Navigation", "type": "liste"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>ap:navigation:waze</t>
+        </is>
+      </c>
+      <c r="B52" s="70" t="inlineStr">
+        <is>
+          <t>Applis proposées par Navigation</t>
+        </is>
+      </c>
+      <c r="C52" s="71" t="inlineStr">
+        <is>
+          <t>Waze</t>
+        </is>
+      </c>
+      <c r="D52" s="71" t="inlineStr">
+        <is>
+          <t>waze://</t>
+        </is>
+      </c>
+      <c r="E52" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.waze;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.waze;end</t>
+        </is>
+      </c>
+      <c r="F52" s="71" t="inlineStr">
+        <is>
+          <t>https://www.waze.com/live-map</t>
+        </is>
+      </c>
+      <c r="G52" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H52" s="72" t="n"/>
+      <c r="I52" s="72" t="n"/>
+      <c r="J52" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Waze", "store": "Waze", "app": "waze://", "web": "https://www.waze.com/live-map", "android": "intent://#Intent;package=com.waze;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.waze;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>ap:navigation:plans</t>
+        </is>
+      </c>
+      <c r="B53" s="70" t="inlineStr">
+        <is>
+          <t>Applis proposées par Navigation</t>
+        </is>
+      </c>
+      <c r="C53" s="71" t="inlineStr">
+        <is>
+          <t>Plans</t>
+        </is>
+      </c>
+      <c r="D53" s="71" t="inlineStr">
+        <is>
+          <t>maps://</t>
+        </is>
+      </c>
+      <c r="E53" s="71" t="n"/>
+      <c r="F53" s="71" t="inlineStr">
+        <is>
+          <t>https://maps.apple.com</t>
+        </is>
+      </c>
+      <c r="G53" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H53" s="72" t="n"/>
+      <c r="I53" s="72" t="inlineStr">
+        <is>
+          <t>pas d'Apple Plans sur Android : Google Maps prend le relais</t>
+        </is>
+      </c>
+      <c r="J53" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Plans", "storeId": "915056765", "app": "maps://", "web": "https://maps.apple.com"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" outlineLevel="1" ht="15" customHeight="1" s="40">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>ap:navigation:google-maps</t>
+        </is>
+      </c>
+      <c r="B54" s="70" t="inlineStr">
+        <is>
+          <t>Applis proposées par Navigation</t>
+        </is>
+      </c>
+      <c r="C54" s="71" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="D54" s="71" t="inlineStr">
+        <is>
+          <t>comgooglemaps://</t>
+        </is>
+      </c>
+      <c r="E54" s="71" t="inlineStr">
+        <is>
+          <t>intent://#Intent;package=com.google.android.apps.maps;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.maps;end</t>
+        </is>
+      </c>
+      <c r="F54" s="71" t="inlineStr">
+        <is>
+          <t>https://maps.google.com</t>
+        </is>
+      </c>
+      <c r="G54" s="69" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H54" s="72" t="n"/>
+      <c r="I54" s="72" t="n"/>
+      <c r="J54" s="39" t="inlineStr">
+        <is>
+          <t>{"support": "ok", "def": {"label": "Google Maps", "store": "Google Maps", "app": "comgooglemaps://", "web": "https://maps.google.com", "android": "intent://#Intent;package=com.google.android.apps.maps;S.browser_fallback_url=https%3A%2F%2Fplay.google.com%2Fstore%2Fapps%2Fdetails%3Fid%3Dcom.google.android.apps.maps;end"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57" ht="15" customHeight="1" s="40">
+      <c r="B57" s="73" t="inlineStr">
+        <is>
+          <t>MES AJOUTS — tape ce que tu veux ajouter : la tâche essaie de le récupérer et écrit le résultat (✅ / ⚠️ / ❌) dans la colonne « Résultat »</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1" s="40">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Dossier (Finance, Travail… ou nouveau)</t>
+        </is>
+      </c>
+      <c r="C58" s="74" t="inlineStr">
+        <is>
+          <t>Nom de l'appli</t>
+        </is>
+      </c>
+      <c r="D58" s="74" t="inlineStr">
+        <is>
+          <t>Lien iPhone (ex. spotify://)</t>
+        </is>
+      </c>
+      <c r="G58" s="74" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H58" s="74" t="inlineStr">
+        <is>
+          <t>Résultat</t>
+        </is>
+      </c>
+      <c r="I58" s="74" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="40">
+      <c r="A59" s="39" t="inlineStr">
+        <is>
+          <t>exemple</t>
+        </is>
+      </c>
+      <c r="B59" s="75" t="inlineStr">
+        <is>
+          <t>Écran d'accueil (dossiers et pages)</t>
+        </is>
+      </c>
+      <c r="C59" s="75" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="D59" s="75" t="inlineStr">
+        <is>
+          <t>spotify://</t>
+        </is>
+      </c>
+      <c r="G59" s="75" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I59" s="75" t="inlineStr">
+        <is>
+          <t>Ligne d'exemple : ignorée par la tâche</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="40">
+      <c r="A60" s="39" t="inlineStr">
+        <is>
+          <t>ajout:1</t>
+        </is>
+      </c>
+      <c r="B60" s="76" t="n"/>
+      <c r="C60" s="76" t="n"/>
+      <c r="D60" s="76" t="n"/>
+      <c r="G60" s="77" t="n"/>
+    </row>
+    <row r="61" ht="15" customHeight="1" s="40">
+      <c r="A61" s="39" t="inlineStr">
+        <is>
+          <t>ajout:2</t>
+        </is>
+      </c>
+      <c r="B61" s="76" t="n"/>
+      <c r="C61" s="76" t="n"/>
+      <c r="D61" s="76" t="n"/>
+      <c r="G61" s="77" t="n"/>
+    </row>
+    <row r="62" ht="15" customHeight="1" s="40">
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>ajout:3</t>
+        </is>
+      </c>
+      <c r="B62" s="76" t="n"/>
+      <c r="C62" s="76" t="n"/>
+      <c r="D62" s="76" t="n"/>
+      <c r="G62" s="77" t="n"/>
+    </row>
+    <row r="63" ht="15" customHeight="1" s="40">
+      <c r="A63" s="39" t="inlineStr">
+        <is>
+          <t>ajout:4</t>
+        </is>
+      </c>
+      <c r="B63" s="76" t="n"/>
+      <c r="C63" s="76" t="n"/>
+      <c r="D63" s="76" t="n"/>
+      <c r="G63" s="77" t="n"/>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="40">
+      <c r="A64" s="39" t="inlineStr">
+        <is>
+          <t>ajout:5</t>
+        </is>
+      </c>
+      <c r="B64" s="76" t="n"/>
+      <c r="C64" s="76" t="n"/>
+      <c r="D64" s="76" t="n"/>
+      <c r="G64" s="77" t="n"/>
+    </row>
+    <row r="65" ht="15" customHeight="1" s="40">
+      <c r="A65" s="39" t="inlineStr">
+        <is>
+          <t>ajout:6</t>
+        </is>
+      </c>
+      <c r="B65" s="76" t="n"/>
+      <c r="C65" s="76" t="n"/>
+      <c r="D65" s="76" t="n"/>
+      <c r="G65" s="77" t="n"/>
+    </row>
+    <row r="66" ht="15" customHeight="1" s="40">
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>ajout:7</t>
+        </is>
+      </c>
+      <c r="B66" s="76" t="n"/>
+      <c r="C66" s="76" t="n"/>
+      <c r="D66" s="76" t="n"/>
+      <c r="G66" s="77" t="n"/>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="40">
+      <c r="A67" s="39" t="inlineStr">
+        <is>
+          <t>ajout:8</t>
+        </is>
+      </c>
+      <c r="B67" s="76" t="n"/>
+      <c r="C67" s="76" t="n"/>
+      <c r="D67" s="76" t="n"/>
+      <c r="G67" s="77" t="n"/>
+    </row>
+    <row r="68" ht="15" customHeight="1" s="40">
+      <c r="A68" s="39" t="inlineStr">
+        <is>
+          <t>ajout:9</t>
+        </is>
+      </c>
+      <c r="B68" s="76" t="n"/>
+      <c r="C68" s="76" t="n"/>
+      <c r="D68" s="76" t="n"/>
+      <c r="G68" s="77" t="n"/>
+    </row>
+    <row r="69" ht="15" customHeight="1" s="40">
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>ajout:10</t>
+        </is>
+      </c>
+      <c r="B69" s="76" t="n"/>
+      <c r="C69" s="76" t="n"/>
+      <c r="D69" s="76" t="n"/>
+      <c r="G69" s="77" t="n"/>
+    </row>
+    <row r="70" ht="15" customHeight="1" s="40">
+      <c r="A70" s="39" t="inlineStr">
+        <is>
+          <t>ajout:11</t>
+        </is>
+      </c>
+      <c r="B70" s="76" t="n"/>
+      <c r="C70" s="76" t="n"/>
+      <c r="D70" s="76" t="n"/>
+      <c r="G70" s="77" t="n"/>
+    </row>
+    <row r="71" ht="15" customHeight="1" s="40">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>ajout:12</t>
+        </is>
+      </c>
+      <c r="B71" s="76" t="n"/>
+      <c r="C71" s="76" t="n"/>
+      <c r="D71" s="76" t="n"/>
+      <c r="G71" s="77" t="n"/>
+    </row>
+    <row r="72" ht="15" customHeight="1" s="40">
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>ajout:13</t>
+        </is>
+      </c>
+      <c r="B72" s="76" t="n"/>
+      <c r="C72" s="76" t="n"/>
+      <c r="D72" s="76" t="n"/>
+      <c r="G72" s="77" t="n"/>
+    </row>
+    <row r="73" ht="15" customHeight="1" s="40">
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>ajout:14</t>
+        </is>
+      </c>
+      <c r="B73" s="76" t="n"/>
+      <c r="C73" s="76" t="n"/>
+      <c r="D73" s="76" t="n"/>
+      <c r="G73" s="77" t="n"/>
+    </row>
+    <row r="74" ht="15" customHeight="1" s="40">
+      <c r="A74" s="39" t="inlineStr">
+        <is>
+          <t>ajout:15</t>
+        </is>
+      </c>
+      <c r="B74" s="76" t="n"/>
+      <c r="C74" s="76" t="n"/>
+      <c r="D74" s="76" t="n"/>
+      <c r="G74" s="77" t="n"/>
+    </row>
+    <row r="75" ht="15" customHeight="1" s="40">
+      <c r="A75" s="39" t="inlineStr">
+        <is>
+          <t>ajout:16</t>
+        </is>
+      </c>
+      <c r="B75" s="76" t="n"/>
+      <c r="C75" s="76" t="n"/>
+      <c r="D75" s="76" t="n"/>
+      <c r="G75" s="77" t="n"/>
+    </row>
+    <row r="76" ht="15" customHeight="1" s="40">
+      <c r="A76" s="39" t="inlineStr">
+        <is>
+          <t>ajout:17</t>
+        </is>
+      </c>
+      <c r="B76" s="76" t="n"/>
+      <c r="C76" s="76" t="n"/>
+      <c r="D76" s="76" t="n"/>
+      <c r="G76" s="77" t="n"/>
+    </row>
+    <row r="77" ht="15" customHeight="1" s="40">
+      <c r="A77" s="39" t="inlineStr">
+        <is>
+          <t>ajout:18</t>
+        </is>
+      </c>
+      <c r="B77" s="76" t="n"/>
+      <c r="C77" s="76" t="n"/>
+      <c r="D77" s="76" t="n"/>
+      <c r="G77" s="77" t="n"/>
+    </row>
+    <row r="78" ht="15" customHeight="1" s="40">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>ajout:19</t>
+        </is>
+      </c>
+      <c r="B78" s="76" t="n"/>
+      <c r="C78" s="76" t="n"/>
+      <c r="D78" s="76" t="n"/>
+      <c r="G78" s="77" t="n"/>
+    </row>
+    <row r="79" ht="15" customHeight="1" s="40">
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>ajout:20</t>
+        </is>
+      </c>
+      <c r="B79" s="76" t="n"/>
+      <c r="C79" s="76" t="n"/>
+      <c r="D79" s="76" t="n"/>
+      <c r="G79" s="77" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="B5:I54"/>
+  <mergeCells count="4">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B57:I57"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6:I54">
+    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
+      <formula>$G6="Oui"</formula>
+    </cfRule>
+    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="11" text="" percent="0" bottom="0">
+      <formula>$G6="Non"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G6:G79" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choix" error="Réponds « Oui », « Non » ou laisse vide." type="list" errorStyle="stop" operator="between">
+      <formula1>"Oui,Non"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <tabColor rgb="FF274C77"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="1"/>
   <cols>
@@ -7611,7 +10233,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=apparence;version=1</t>
+          <t>module=apparence;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -8793,7 +11415,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=sport;version=1</t>
+          <t>module=sport;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -9004,7 +11626,7 @@
       <c r="K8" s="72" t="n"/>
       <c r="L8" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "fra.2", "region": "fr", "flag": "🇫🇷", "sport": "soccer", "group": "foot", "name": "Ligue 2", "tv": ["beIN Sports"], "rounds": true, "of": "fr.2", "tsdb": {"c": "France", "s": "Soccer", "re": {}}}}</t>
+          <t>{"support": "ok", "def": {"id": "fra.2", "region": "fr", "flag": "🇫🇷", "sport": "soccer", "group": "foot", "name": "Ligue 2", "tv": ["beIN Sports"], "rounds": true, "of": "fr.2", "tsdb": {"c": "France", "s": "Soccer", "re": {"re": "ligue 2", "flags": "i"}}}}</t>
         </is>
       </c>
     </row>
@@ -11556,7 +14178,7 @@
       <c r="K64" s="72" t="n"/>
       <c r="L64" s="39" t="inlineStr">
         <is>
-          <t>{"support": "ok", "def": {"id": "270559", "region": "rfr", "flag": "🇫🇷", "sport": "rugby", "group": "rugby", "name": "Top 14", "tv": ["Canal+"], "rounds": true, "tsdb": {"c": "France", "s": "Rugby", "re": {}}, "badges": true}}</t>
+          <t>{"support": "ok", "def": {"id": "270559", "region": "rfr", "flag": "🇫🇷", "sport": "rugby", "group": "rugby", "name": "Top 14", "tv": ["Canal+"], "rounds": true, "tsdb": {"c": "France", "s": "Rugby", "re": {"re": "top ?14", "flags": "i"}}, "badges": true}}</t>
         </is>
       </c>
     </row>
@@ -16089,7 +18711,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=equipes;version=1</t>
+          <t>module=equipes;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -18008,7 +20630,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=actus;version=1</t>
+          <t>module=actus;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -26681,7 +29303,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=actus-en;version=1</t>
+          <t>module=actus-en;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -30697,7 +33319,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=marches;version=1</t>
+          <t>module=marches;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -34094,7 +36716,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=videos;version=1</t>
+          <t>module=videos;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">
@@ -35407,7 +38029,7 @@
     <row r="1" ht="30" customHeight="1" s="40">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>module=youtube;version=1</t>
+          <t>module=youtube;version=2</t>
         </is>
       </c>
       <c r="B1" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Configuration depuis le classeur
</commit_message>
<xml_diff>
--- a/config/configuration-resultat.xlsx
+++ b/config/configuration-resultat.xlsx
@@ -744,7 +744,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -1296,7 +1296,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -3263,7 +3263,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -3985,7 +3985,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J79"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -6333,7 +6333,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -6852,7 +6852,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -7509,7 +7509,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K182"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -14647,7 +14647,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I256"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -23323,7 +23323,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I130"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -27337,7 +27337,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K108"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -27638,11 +27638,15 @@
       </c>
       <c r="E11" s="23" t="n"/>
       <c r="F11" s="23" t="n"/>
-      <c r="G11" s="21" t="n"/>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="H11" s="21" t="n"/>
       <c r="I11" s="24" t="inlineStr">
         <is>
-          <t>à vérifier</t>
+          <t>⚠️ non testé : site injoignable pour l'instant (HTTPError) — gardé, nouvel essai au prochain dépôt</t>
         </is>
       </c>
       <c r="J11" s="24" t="n"/>
@@ -30732,7 +30736,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -32012,7 +32016,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H85"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -34214,7 +34218,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H108"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col hidden="1" width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>

</xml_diff>